<commit_message>
Update models and pitches
</commit_message>
<xml_diff>
--- a/public/pitches/APP_vf.xlsx
+++ b/public/pitches/APP_vf.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\itsme\OneDrive\Documents\LSE\Sipher street\AppLoving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF3D59CD-B797-4D88-9FB4-CA4E8FB35CA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BAD1E0B-4CF8-439B-9F7F-67EC7DDC49DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{6C93F160-F9EC-42EA-8764-3FE5C2237C03}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6C93F160-F9EC-42EA-8764-3FE5C2237C03}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="6" r:id="rId1"/>
@@ -20,9 +20,8 @@
     <sheet name="DCF" sheetId="9" r:id="rId5"/>
     <sheet name="WACC" sheetId="8" r:id="rId6"/>
     <sheet name="Income Statement" sheetId="1" r:id="rId7"/>
-    <sheet name="Graphs" sheetId="10" r:id="rId8"/>
-    <sheet name="Balance Sheet" sheetId="2" r:id="rId9"/>
-    <sheet name="Cash Flow" sheetId="3" r:id="rId10"/>
+    <sheet name="Balance Sheet" sheetId="2" r:id="rId8"/>
+    <sheet name="Cash Flow" sheetId="3" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="CaseSel">'Metrics &amp; Drivers'!$D$3</definedName>
@@ -97,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="228">
   <si>
     <t>AppLovin Corp (APP.O)</t>
   </si>
@@ -781,22 +780,13 @@
   </si>
   <si>
     <t>AppLovin Share Price ($)</t>
-  </si>
-  <si>
-    <t>Revenue ($M)</t>
-  </si>
-  <si>
-    <t>Net Income ($M)</t>
-  </si>
-  <si>
-    <t>Net Margin %</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="12">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="#,##0.0;\(#,##0.0\);&quot;—&quot;"/>
     <numFmt numFmtId="166" formatCode="#,##0.00;\(#,##0.00\);&quot;—&quot;"/>
@@ -807,10 +797,9 @@
     <numFmt numFmtId="171" formatCode="&quot;£&quot;#,##0.00"/>
     <numFmt numFmtId="172" formatCode="0.0"/>
     <numFmt numFmtId="173" formatCode="0.0\x"/>
-    <numFmt numFmtId="174" formatCode="#,##0.0;\(#,##0.0\)"/>
     <numFmt numFmtId="175" formatCode="[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="45" x14ac:knownFonts="1">
+  <fonts count="40" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -840,57 +829,67 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Garamond"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Garamond"/>
+      <family val="1"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Garamond"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Garamond"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Garamond"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Garamond"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="13"/>
       <color theme="1"/>
       <name val="Garamond"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF008000"/>
       <name val="Garamond"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="13"/>
       <color rgb="FF000000"/>
       <name val="Garamond"/>
+      <family val="1"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Garamond"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="11"/>
@@ -902,6 +901,7 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Garamond"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
@@ -909,18 +909,21 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Garamond"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF008000"/>
       <name val="Garamond"/>
+      <family val="1"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Garamond"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="11"/>
@@ -933,6 +936,7 @@
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Garamond"/>
+      <family val="1"/>
     </font>
     <font>
       <i/>
@@ -1060,37 +1064,8 @@
       <name val="Garamond"/>
       <family val="2"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF1E90FF"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF333333"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF00CED1"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF8C00"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
-  <fills count="12">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1143,20 +1118,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF333333"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF5F5F5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="62">
+  <borders count="55">
     <border>
       <left/>
       <right/>
@@ -1750,79 +1713,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF555555"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFDDDDDD"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFDDDDDD"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF555555"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF999999"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF999999"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF555555"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF999999"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FFDDDDDD"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF999999"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FFDDDDDD"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF555555"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1831,7 +1721,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="239">
+  <cellXfs count="226">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2345,6 +2235,9 @@
     <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
+    <xf numFmtId="175" fontId="31" fillId="6" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="26" fillId="3" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2356,42 +2249,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="40" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="11" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="42" fillId="11" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="7" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="42" fillId="7" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="174" fontId="42" fillId="7" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="11" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="42" fillId="11" borderId="57" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="10" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="42" fillId="11" borderId="59" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="42" fillId="7" borderId="60" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="42" fillId="11" borderId="61" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="31" fillId="6" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -2856,10 +2713,10 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="438" row="1">
+  <wetp:taskpane dockstate="right" visibility="1" width="350" row="0">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
-  <wetp:taskpane dockstate="right" visibility="0" width="438" row="1">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="2">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -2957,1210 +2814,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1B8D43B-0AE5-451E-8577-8383133CC245}">
-  <dimension ref="B2:I53"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="1.88671875" customWidth="1"/>
-    <col min="2" max="2" width="46.33203125" customWidth="1"/>
-    <col min="3" max="9" width="15.77734375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:9" ht="17.399999999999999" x14ac:dyDescent="0.35">
-      <c r="B2" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-    </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B3" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-    </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-    </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-    </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B6" s="2"/>
-      <c r="C6" s="224" t="s">
-        <v>117</v>
-      </c>
-      <c r="D6" s="224"/>
-      <c r="E6" s="224"/>
-      <c r="F6" s="224"/>
-      <c r="G6" s="224"/>
-      <c r="H6" s="224"/>
-      <c r="I6" s="224"/>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B7" s="216"/>
-      <c r="C7" s="216">
-        <v>2019</v>
-      </c>
-      <c r="D7" s="216">
-        <v>2020</v>
-      </c>
-      <c r="E7" s="216">
-        <v>2021</v>
-      </c>
-      <c r="F7" s="216">
-        <v>2022</v>
-      </c>
-      <c r="G7" s="216">
-        <v>2023</v>
-      </c>
-      <c r="H7" s="216">
-        <v>2024</v>
-      </c>
-      <c r="I7" s="216">
-        <v>2025</v>
-      </c>
-    </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B8" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-    </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B9" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C9" s="16">
-        <f>'Income Statement'!C29</f>
-        <v>118.99999999999994</v>
-      </c>
-      <c r="D9" s="16">
-        <f>'Income Statement'!D29</f>
-        <v>-43.320000000000192</v>
-      </c>
-      <c r="E9" s="16">
-        <f>'Income Statement'!E29</f>
-        <v>35.29999999999977</v>
-      </c>
-      <c r="F9" s="16">
-        <f>'Income Statement'!F29</f>
-        <v>-192.98999999999998</v>
-      </c>
-      <c r="G9" s="16">
-        <f>'Income Statement'!G29</f>
-        <v>356.66999999999979</v>
-      </c>
-      <c r="H9" s="16">
-        <f>'Income Statement'!H29</f>
-        <v>1579.83</v>
-      </c>
-      <c r="I9" s="16">
-        <f>'Income Statement'!I29</f>
-        <v>3333.77</v>
-      </c>
-    </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B10" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-    </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B11" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C11" s="6">
-        <v>92.81</v>
-      </c>
-      <c r="D11" s="6">
-        <v>255</v>
-      </c>
-      <c r="E11" s="6">
-        <v>431.1</v>
-      </c>
-      <c r="F11" s="6">
-        <v>547.1</v>
-      </c>
-      <c r="G11" s="6">
-        <v>489</v>
-      </c>
-      <c r="H11" s="6">
-        <v>448.7</v>
-      </c>
-      <c r="I11" s="6">
-        <v>194.8</v>
-      </c>
-    </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B12" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C12" s="6">
-        <v>10.220000000000001</v>
-      </c>
-      <c r="D12" s="6">
-        <v>62.39</v>
-      </c>
-      <c r="E12" s="6">
-        <v>133.19999999999999</v>
-      </c>
-      <c r="F12" s="6">
-        <v>191.6</v>
-      </c>
-      <c r="G12" s="6">
-        <v>363.1</v>
-      </c>
-      <c r="H12" s="6">
-        <v>369.4</v>
-      </c>
-      <c r="I12" s="6">
-        <v>210.4</v>
-      </c>
-    </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B13" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C13" s="6">
-        <v>4.9800000000000004</v>
-      </c>
-      <c r="D13" s="6">
-        <v>8.15</v>
-      </c>
-      <c r="E13" s="6">
-        <v>12.83</v>
-      </c>
-      <c r="F13" s="6">
-        <v>12.68</v>
-      </c>
-      <c r="G13" s="6">
-        <v>9.36</v>
-      </c>
-      <c r="H13" s="6">
-        <v>5.46</v>
-      </c>
-      <c r="I13" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B14" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C14" s="6">
-        <v>0</v>
-      </c>
-      <c r="D14" s="6">
-        <v>0</v>
-      </c>
-      <c r="E14" s="6">
-        <v>0</v>
-      </c>
-      <c r="F14" s="6">
-        <v>0</v>
-      </c>
-      <c r="G14" s="6">
-        <v>0</v>
-      </c>
-      <c r="H14" s="6">
-        <v>0</v>
-      </c>
-      <c r="I14" s="6">
-        <v>188.9</v>
-      </c>
-    </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B15" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C15" s="6">
-        <v>0</v>
-      </c>
-      <c r="D15" s="6">
-        <v>0</v>
-      </c>
-      <c r="E15" s="6">
-        <v>0</v>
-      </c>
-      <c r="F15" s="6">
-        <v>0</v>
-      </c>
-      <c r="G15" s="6">
-        <v>0</v>
-      </c>
-      <c r="H15" s="6">
-        <v>0</v>
-      </c>
-      <c r="I15" s="6">
-        <v>-106.2</v>
-      </c>
-    </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B16" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C16" s="6">
-        <v>0</v>
-      </c>
-      <c r="D16" s="6">
-        <v>0</v>
-      </c>
-      <c r="E16" s="6">
-        <v>0</v>
-      </c>
-      <c r="F16" s="6">
-        <v>0</v>
-      </c>
-      <c r="G16" s="6">
-        <v>27.95</v>
-      </c>
-      <c r="H16" s="6">
-        <v>0</v>
-      </c>
-      <c r="I16" s="6">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B17" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C17" s="6">
-        <v>0</v>
-      </c>
-      <c r="D17" s="6">
-        <v>0</v>
-      </c>
-      <c r="E17" s="6">
-        <v>0</v>
-      </c>
-      <c r="F17" s="6">
-        <v>127.9</v>
-      </c>
-      <c r="G17" s="6">
-        <v>0</v>
-      </c>
-      <c r="H17" s="6">
-        <v>1.65</v>
-      </c>
-      <c r="I17" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B18" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C18" s="6">
-        <v>0</v>
-      </c>
-      <c r="D18" s="6">
-        <v>0</v>
-      </c>
-      <c r="E18" s="6">
-        <v>18.239999999999998</v>
-      </c>
-      <c r="F18" s="6">
-        <v>0</v>
-      </c>
-      <c r="G18" s="6">
-        <v>0</v>
-      </c>
-      <c r="H18" s="6">
-        <v>28.38</v>
-      </c>
-      <c r="I18" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B19" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C19" s="6">
-        <v>2.69</v>
-      </c>
-      <c r="D19" s="6">
-        <v>7.68</v>
-      </c>
-      <c r="E19" s="6">
-        <v>15.58</v>
-      </c>
-      <c r="F19" s="6">
-        <v>18.91</v>
-      </c>
-      <c r="G19" s="6">
-        <v>24.13</v>
-      </c>
-      <c r="H19" s="6">
-        <v>15.06</v>
-      </c>
-      <c r="I19" s="6">
-        <v>21.46</v>
-      </c>
-    </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B20" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B21" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C21" s="6">
-        <v>-33.520000000000003</v>
-      </c>
-      <c r="D21" s="6">
-        <v>-113.2</v>
-      </c>
-      <c r="E21" s="6">
-        <v>-202</v>
-      </c>
-      <c r="F21" s="6">
-        <v>-174.8</v>
-      </c>
-      <c r="G21" s="6">
-        <v>-261.3</v>
-      </c>
-      <c r="H21" s="6">
-        <v>-467</v>
-      </c>
-      <c r="I21" s="6">
-        <v>-542.20000000000005</v>
-      </c>
-    </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B22" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C22" s="6">
-        <v>-21.35</v>
-      </c>
-      <c r="D22" s="6">
-        <v>-32.380000000000003</v>
-      </c>
-      <c r="E22" s="6">
-        <v>-143.26</v>
-      </c>
-      <c r="F22" s="6">
-        <v>-81.06</v>
-      </c>
-      <c r="G22" s="6">
-        <v>-133.97999999999999</v>
-      </c>
-      <c r="H22" s="6">
-        <v>-185.34</v>
-      </c>
-      <c r="I22" s="6">
-        <v>134.69999999999999</v>
-      </c>
-    </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B23" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C23" s="6">
-        <v>13.53</v>
-      </c>
-      <c r="D23" s="6">
-        <v>49.12</v>
-      </c>
-      <c r="E23" s="6">
-        <v>98.61</v>
-      </c>
-      <c r="F23" s="6">
-        <v>3.48</v>
-      </c>
-      <c r="G23" s="6">
-        <v>98.57</v>
-      </c>
-      <c r="H23" s="6">
-        <v>189.6</v>
-      </c>
-      <c r="I23" s="6">
-        <v>232.5</v>
-      </c>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B24" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C24" s="6">
-        <v>5.66</v>
-      </c>
-      <c r="D24" s="6">
-        <v>2.78</v>
-      </c>
-      <c r="E24" s="6">
-        <v>3.06</v>
-      </c>
-      <c r="F24" s="6">
-        <v>-6.41</v>
-      </c>
-      <c r="G24" s="6">
-        <v>92.75</v>
-      </c>
-      <c r="H24" s="6">
-        <v>134</v>
-      </c>
-      <c r="I24" s="6">
-        <v>268.2</v>
-      </c>
-    </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B25" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="C25" s="6">
-        <v>6.72</v>
-      </c>
-      <c r="D25" s="6">
-        <v>35.49</v>
-      </c>
-      <c r="E25" s="6">
-        <v>-13.91</v>
-      </c>
-      <c r="F25" s="6">
-        <v>-14.71</v>
-      </c>
-      <c r="G25" s="6">
-        <v>13.86</v>
-      </c>
-      <c r="H25" s="6">
-        <v>-6.63</v>
-      </c>
-      <c r="I25" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B26" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C26" s="6">
-        <v>-2.2400000000000002</v>
-      </c>
-      <c r="D26" s="6">
-        <v>-8.81</v>
-      </c>
-      <c r="E26" s="6">
-        <v>-26.85</v>
-      </c>
-      <c r="F26" s="6">
-        <v>-18.899999999999999</v>
-      </c>
-      <c r="G26" s="6">
-        <v>-18.61</v>
-      </c>
-      <c r="H26" s="6">
-        <v>-14.11</v>
-      </c>
-      <c r="I26" s="6">
-        <v>-15.23</v>
-      </c>
-    </row>
-    <row r="27" spans="2:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="C27" s="7">
-        <f>C9+SUM(C11:C19)+SUM(C21:C26)</f>
-        <v>198.49999999999991</v>
-      </c>
-      <c r="D27" s="7">
-        <f t="shared" ref="D27:I27" si="0">D9+SUM(D11:D19)+SUM(D21:D26)</f>
-        <v>222.89999999999975</v>
-      </c>
-      <c r="E27" s="7">
-        <f t="shared" si="0"/>
-        <v>361.89999999999975</v>
-      </c>
-      <c r="F27" s="7">
-        <f t="shared" si="0"/>
-        <v>412.79999999999995</v>
-      </c>
-      <c r="G27" s="7">
-        <f t="shared" si="0"/>
-        <v>1061.4999999999998</v>
-      </c>
-      <c r="H27" s="7">
-        <f t="shared" si="0"/>
-        <v>2098.9999999999995</v>
-      </c>
-      <c r="I27" s="7">
-        <f t="shared" si="0"/>
-        <v>3971.1</v>
-      </c>
-    </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B28" s="2"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="8"/>
-      <c r="I28" s="8"/>
-    </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B29" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
-      <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
-      <c r="H29" s="8"/>
-      <c r="I29" s="8"/>
-    </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B30" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C30" s="6">
-        <v>-404.2</v>
-      </c>
-      <c r="D30" s="6">
-        <v>-674.7</v>
-      </c>
-      <c r="E30" s="6">
-        <v>-1206.5</v>
-      </c>
-      <c r="F30" s="6">
-        <v>-1339.8</v>
-      </c>
-      <c r="G30" s="6">
-        <v>0</v>
-      </c>
-      <c r="H30" s="6">
-        <v>0</v>
-      </c>
-      <c r="I30" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B31" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C31" s="6">
-        <v>-3.36</v>
-      </c>
-      <c r="D31" s="6">
-        <v>-3.24</v>
-      </c>
-      <c r="E31" s="6">
-        <v>-1.39</v>
-      </c>
-      <c r="F31" s="6">
-        <v>-0.66</v>
-      </c>
-      <c r="G31" s="6">
-        <v>-4.25</v>
-      </c>
-      <c r="H31" s="6">
-        <v>-4.78</v>
-      </c>
-      <c r="I31" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B32" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="C32" s="6">
-        <v>0</v>
-      </c>
-      <c r="D32" s="6">
-        <v>0</v>
-      </c>
-      <c r="E32" s="6">
-        <v>-4.07</v>
-      </c>
-      <c r="F32" s="6">
-        <v>-5.95</v>
-      </c>
-      <c r="G32" s="6">
-        <v>-63.9</v>
-      </c>
-      <c r="H32" s="6">
-        <v>-25.55</v>
-      </c>
-      <c r="I32" s="6">
-        <v>-28.32</v>
-      </c>
-    </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B33" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="C33" s="6">
-        <v>-4</v>
-      </c>
-      <c r="D33" s="6">
-        <v>-2</v>
-      </c>
-      <c r="E33" s="6">
-        <v>-15</v>
-      </c>
-      <c r="F33" s="6">
-        <v>-66.34</v>
-      </c>
-      <c r="G33" s="6">
-        <v>-17.93</v>
-      </c>
-      <c r="H33" s="6">
-        <v>-76.98</v>
-      </c>
-      <c r="I33" s="6">
-        <v>-20.18</v>
-      </c>
-    </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B34" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="C34" s="6">
-        <v>0</v>
-      </c>
-      <c r="D34" s="6">
-        <v>0</v>
-      </c>
-      <c r="E34" s="6">
-        <v>12.01</v>
-      </c>
-      <c r="F34" s="6">
-        <v>41.31</v>
-      </c>
-      <c r="G34" s="6">
-        <v>8.25</v>
-      </c>
-      <c r="H34" s="6">
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="I34" s="6">
-        <v>407.3</v>
-      </c>
-    </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B35" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="C35" s="6">
-        <v>-0.04</v>
-      </c>
-      <c r="D35" s="6">
-        <v>0.04</v>
-      </c>
-      <c r="E35" s="6">
-        <v>0.05</v>
-      </c>
-      <c r="F35" s="6">
-        <v>-0.06</v>
-      </c>
-      <c r="G35" s="6">
-        <v>0</v>
-      </c>
-      <c r="H35" s="6">
-        <v>-0.05</v>
-      </c>
-      <c r="I35" s="6">
-        <v>-0.4</v>
-      </c>
-    </row>
-    <row r="36" spans="2:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="C36" s="7">
-        <f>SUM(C30:C35)</f>
-        <v>-411.6</v>
-      </c>
-      <c r="D36" s="7">
-        <f t="shared" ref="D36:I36" si="1">SUM(D30:D35)</f>
-        <v>-679.90000000000009</v>
-      </c>
-      <c r="E36" s="7">
-        <f t="shared" si="1"/>
-        <v>-1214.9000000000001</v>
-      </c>
-      <c r="F36" s="7">
-        <f t="shared" si="1"/>
-        <v>-1371.5</v>
-      </c>
-      <c r="G36" s="7">
-        <f t="shared" si="1"/>
-        <v>-77.830000000000013</v>
-      </c>
-      <c r="H36" s="7">
-        <f t="shared" si="1"/>
-        <v>-106.8</v>
-      </c>
-      <c r="I36" s="7">
-        <f t="shared" si="1"/>
-        <v>358.40000000000003</v>
-      </c>
-    </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B37" s="2"/>
-      <c r="C37" s="8"/>
-      <c r="D37" s="8"/>
-      <c r="E37" s="8"/>
-      <c r="F37" s="8"/>
-      <c r="G37" s="8"/>
-      <c r="H37" s="8"/>
-      <c r="I37" s="8"/>
-    </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B38" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C38" s="8"/>
-      <c r="D38" s="8"/>
-      <c r="E38" s="8"/>
-      <c r="F38" s="8"/>
-      <c r="G38" s="8"/>
-      <c r="H38" s="8"/>
-      <c r="I38" s="8"/>
-    </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B39" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="C39" s="6">
-        <v>388.9</v>
-      </c>
-      <c r="D39" s="6">
-        <v>481.3</v>
-      </c>
-      <c r="E39" s="6">
-        <v>2329.1</v>
-      </c>
-      <c r="F39" s="6">
-        <v>0</v>
-      </c>
-      <c r="G39" s="6">
-        <v>395.3</v>
-      </c>
-      <c r="H39" s="6">
-        <v>4614.8</v>
-      </c>
-      <c r="I39" s="6">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B40" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="C40" s="6">
-        <v>-11.21</v>
-      </c>
-      <c r="D40" s="6">
-        <v>-64.290000000000006</v>
-      </c>
-      <c r="E40" s="6">
-        <v>-719.8</v>
-      </c>
-      <c r="F40" s="6">
-        <v>-25.81</v>
-      </c>
-      <c r="G40" s="6">
-        <v>-498</v>
-      </c>
-      <c r="H40" s="6">
-        <v>-4225.2</v>
-      </c>
-      <c r="I40" s="6">
-        <v>-200</v>
-      </c>
-    </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B41" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="C41" s="6">
-        <v>-0.01</v>
-      </c>
-      <c r="D41" s="6">
-        <v>-1.77</v>
-      </c>
-      <c r="E41" s="6">
-        <v>0</v>
-      </c>
-      <c r="F41" s="6">
-        <v>-338.9</v>
-      </c>
-      <c r="G41" s="6">
-        <v>-1153.5999999999999</v>
-      </c>
-      <c r="H41" s="6">
-        <v>-981.3</v>
-      </c>
-      <c r="I41" s="6">
-        <v>-2191.9</v>
-      </c>
-    </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B42" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="C42" s="6">
-        <v>0</v>
-      </c>
-      <c r="D42" s="6">
-        <v>0</v>
-      </c>
-      <c r="E42" s="6">
-        <v>0</v>
-      </c>
-      <c r="F42" s="6">
-        <v>-27.53</v>
-      </c>
-      <c r="G42" s="6">
-        <v>-246.4</v>
-      </c>
-      <c r="H42" s="6">
-        <v>-1143.5</v>
-      </c>
-      <c r="I42" s="6">
-        <v>-392.4</v>
-      </c>
-    </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B43" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C43" s="6">
-        <v>2.64</v>
-      </c>
-      <c r="D43" s="6">
-        <v>11.62</v>
-      </c>
-      <c r="E43" s="6">
-        <v>1779.24</v>
-      </c>
-      <c r="F43" s="6">
-        <v>31.02</v>
-      </c>
-      <c r="G43" s="6">
-        <v>25.79</v>
-      </c>
-      <c r="H43" s="6">
-        <v>41.8</v>
-      </c>
-      <c r="I43" s="6">
-        <v>25.33</v>
-      </c>
-    </row>
-    <row r="44" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B44" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="C44" s="6">
-        <v>-5.66</v>
-      </c>
-      <c r="D44" s="6">
-        <v>-9.7100000000000009</v>
-      </c>
-      <c r="E44" s="6">
-        <v>-15.27</v>
-      </c>
-      <c r="F44" s="6">
-        <v>-24.08</v>
-      </c>
-      <c r="G44" s="6">
-        <v>-20.170000000000002</v>
-      </c>
-      <c r="H44" s="6">
-        <v>-20.87</v>
-      </c>
-      <c r="I44" s="6">
-        <v>-18.670000000000002</v>
-      </c>
-    </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B45" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="C45" s="6">
-        <v>-41.46</v>
-      </c>
-      <c r="D45" s="6">
-        <v>-39.25</v>
-      </c>
-      <c r="E45" s="6">
-        <v>-263.67</v>
-      </c>
-      <c r="F45" s="6">
-        <v>-141.6</v>
-      </c>
-      <c r="G45" s="6">
-        <v>-65.72</v>
-      </c>
-      <c r="H45" s="6">
-        <v>-35.53</v>
-      </c>
-      <c r="I45" s="6">
-        <v>-15.46</v>
-      </c>
-    </row>
-    <row r="46" spans="2:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B46" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="C46" s="7">
-        <f>SUM(C39:C45)</f>
-        <v>333.2</v>
-      </c>
-      <c r="D46" s="7">
-        <f t="shared" ref="D46:I46" si="2">SUM(D39:D45)</f>
-        <v>377.90000000000003</v>
-      </c>
-      <c r="E46" s="7">
-        <f t="shared" si="2"/>
-        <v>3109.6</v>
-      </c>
-      <c r="F46" s="7">
-        <f t="shared" si="2"/>
-        <v>-526.9</v>
-      </c>
-      <c r="G46" s="7">
-        <f t="shared" si="2"/>
-        <v>-1562.8000000000002</v>
-      </c>
-      <c r="H46" s="7">
-        <f t="shared" si="2"/>
-        <v>-1749.7999999999995</v>
-      </c>
-      <c r="I46" s="7">
-        <f t="shared" si="2"/>
-        <v>-2593.1000000000004</v>
-      </c>
-    </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B47" s="2"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="8"/>
-      <c r="E47" s="8"/>
-      <c r="F47" s="8"/>
-      <c r="G47" s="8"/>
-      <c r="H47" s="8"/>
-      <c r="I47" s="8"/>
-    </row>
-    <row r="48" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B48" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="C48" s="6">
-        <v>0.06</v>
-      </c>
-      <c r="D48" s="6">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="E48" s="6">
-        <v>-3.2</v>
-      </c>
-      <c r="F48" s="6">
-        <v>-4.4800000000000004</v>
-      </c>
-      <c r="G48" s="6">
-        <v>0.78</v>
-      </c>
-      <c r="H48" s="6">
-        <v>-3.15</v>
-      </c>
-      <c r="I48" s="6">
-        <v>9.23</v>
-      </c>
-    </row>
-    <row r="49" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B49" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="C49" s="6">
-        <v>0</v>
-      </c>
-      <c r="D49" s="6">
-        <v>0</v>
-      </c>
-      <c r="E49" s="6">
-        <v>0</v>
-      </c>
-      <c r="F49" s="6">
-        <v>0</v>
-      </c>
-      <c r="G49" s="6">
-        <v>0</v>
-      </c>
-      <c r="H49" s="6">
-        <v>0</v>
-      </c>
-      <c r="I49" s="6">
-        <v>44.38</v>
-      </c>
-    </row>
-    <row r="50" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B50" s="2"/>
-      <c r="C50" s="8"/>
-      <c r="D50" s="8"/>
-      <c r="E50" s="8"/>
-      <c r="F50" s="8"/>
-      <c r="G50" s="8"/>
-      <c r="H50" s="8"/>
-      <c r="I50" s="8"/>
-    </row>
-    <row r="51" spans="2:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B51" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="C51" s="7">
-        <f>C27+C36+C46+C48+C49</f>
-        <v>120.15999999999988</v>
-      </c>
-      <c r="D51" s="7">
-        <f t="shared" ref="D51:I51" si="3">D27+D36+D46+D48+D49</f>
-        <v>-78.960000000000306</v>
-      </c>
-      <c r="E51" s="7">
-        <f t="shared" si="3"/>
-        <v>2253.3999999999996</v>
-      </c>
-      <c r="F51" s="7">
-        <f t="shared" si="3"/>
-        <v>-1490.08</v>
-      </c>
-      <c r="G51" s="7">
-        <f t="shared" si="3"/>
-        <v>-578.35000000000048</v>
-      </c>
-      <c r="H51" s="7">
-        <f t="shared" si="3"/>
-        <v>239.25000000000009</v>
-      </c>
-      <c r="I51" s="7">
-        <f t="shared" si="3"/>
-        <v>1790.0099999999998</v>
-      </c>
-    </row>
-    <row r="52" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B52" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="C52" s="6">
-        <v>276.10000000000002</v>
-      </c>
-      <c r="D52" s="6">
-        <v>396.3</v>
-      </c>
-      <c r="E52" s="6">
-        <v>317.2</v>
-      </c>
-      <c r="F52" s="6">
-        <v>2570.5</v>
-      </c>
-      <c r="G52" s="6">
-        <v>1080.5</v>
-      </c>
-      <c r="H52" s="6">
-        <v>502.2</v>
-      </c>
-      <c r="I52" s="6">
-        <v>697</v>
-      </c>
-    </row>
-    <row r="53" spans="2:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B53" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C53" s="7">
-        <f>C52+C51</f>
-        <v>396.25999999999988</v>
-      </c>
-      <c r="D53" s="7">
-        <f t="shared" ref="D53:I53" si="4">D52+D51</f>
-        <v>317.33999999999969</v>
-      </c>
-      <c r="E53" s="7">
-        <f t="shared" si="4"/>
-        <v>2570.5999999999995</v>
-      </c>
-      <c r="F53" s="7">
-        <f t="shared" si="4"/>
-        <v>1080.42</v>
-      </c>
-      <c r="G53" s="7">
-        <f t="shared" si="4"/>
-        <v>502.14999999999952</v>
-      </c>
-      <c r="H53" s="7">
-        <f t="shared" si="4"/>
-        <v>741.45</v>
-      </c>
-      <c r="I53" s="7">
-        <f t="shared" si="4"/>
-        <v>2487.0099999999998</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="C6:I6"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A210D4E-FEA7-47B9-8D87-459D95B6581E}">
   <dimension ref="A2:M23"/>
@@ -8314,11 +6967,11 @@
       <c r="I5" s="203" t="s">
         <v>134</v>
       </c>
-      <c r="K5" s="221" t="s">
+      <c r="K5" s="222" t="s">
         <v>205</v>
       </c>
-      <c r="L5" s="222"/>
-      <c r="M5" s="223"/>
+      <c r="L5" s="223"/>
+      <c r="M5" s="224"/>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.3">
       <c r="D6" s="138"/>
@@ -8719,7 +7372,7 @@
         <v>216</v>
       </c>
       <c r="L18" s="148"/>
-      <c r="M18" s="238">
+      <c r="M18" s="221">
         <f>M16/M17</f>
         <v>590.09140233469361</v>
       </c>
@@ -9811,15 +8464,15 @@
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B6" s="2"/>
-      <c r="C6" s="224" t="s">
+      <c r="C6" s="225" t="s">
         <v>117</v>
       </c>
-      <c r="D6" s="224"/>
-      <c r="E6" s="224"/>
-      <c r="F6" s="224"/>
-      <c r="G6" s="224"/>
-      <c r="H6" s="224"/>
-      <c r="I6" s="224"/>
+      <c r="D6" s="225"/>
+      <c r="E6" s="225"/>
+      <c r="F6" s="225"/>
+      <c r="G6" s="225"/>
+      <c r="H6" s="225"/>
+      <c r="I6" s="225"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B7" s="215"/>
@@ -10690,194 +9343,6 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{164F09BC-C5F6-4C09-A987-ECC40E0193A7}">
-  <dimension ref="B2:M6"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="24.109375" customWidth="1"/>
-    <col min="3" max="13" width="15.77734375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B2" s="225"/>
-      <c r="C2" s="226">
-        <v>2021</v>
-      </c>
-      <c r="D2" s="226">
-        <v>2022</v>
-      </c>
-      <c r="E2" s="226">
-        <v>2023</v>
-      </c>
-      <c r="F2" s="226">
-        <v>2024</v>
-      </c>
-      <c r="G2" s="226">
-        <v>2025</v>
-      </c>
-      <c r="H2" s="234" t="s">
-        <v>124</v>
-      </c>
-      <c r="I2" s="225" t="s">
-        <v>125</v>
-      </c>
-      <c r="J2" s="225" t="s">
-        <v>126</v>
-      </c>
-      <c r="K2" s="225" t="s">
-        <v>127</v>
-      </c>
-      <c r="L2" s="225" t="s">
-        <v>128</v>
-      </c>
-      <c r="M2" s="225" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B3" s="227" t="s">
-        <v>228</v>
-      </c>
-      <c r="C3" s="228">
-        <v>2793.1</v>
-      </c>
-      <c r="D3" s="228">
-        <v>2817.1</v>
-      </c>
-      <c r="E3" s="228">
-        <v>3283.1</v>
-      </c>
-      <c r="F3" s="228">
-        <v>3224.1</v>
-      </c>
-      <c r="G3" s="228">
-        <v>5480.7</v>
-      </c>
-      <c r="H3" s="235">
-        <f>'Metrics &amp; Drivers'!J7</f>
-        <v>6987.892499999999</v>
-      </c>
-      <c r="I3" s="228">
-        <f>'Metrics &amp; Drivers'!K7</f>
-        <v>8664.9866999999995</v>
-      </c>
-      <c r="J3" s="228">
-        <f>'Metrics &amp; Drivers'!L7</f>
-        <v>10397.984039999999</v>
-      </c>
-      <c r="K3" s="228">
-        <f>'Metrics &amp; Drivers'!M7</f>
-        <v>12061.661486399998</v>
-      </c>
-      <c r="L3" s="228">
-        <f>'Metrics &amp; Drivers'!N7</f>
-        <v>13750.294094495999</v>
-      </c>
-      <c r="M3" s="228">
-        <f>'Metrics &amp; Drivers'!O7</f>
-        <v>15262.826444890561</v>
-      </c>
-    </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B4" s="229" t="s">
-        <v>229</v>
-      </c>
-      <c r="C4" s="230">
-        <v>35.299999999999997</v>
-      </c>
-      <c r="D4" s="231">
-        <v>-192.99</v>
-      </c>
-      <c r="E4" s="230">
-        <v>356.67</v>
-      </c>
-      <c r="F4" s="230">
-        <v>1579.83</v>
-      </c>
-      <c r="G4" s="230">
-        <v>3333.77</v>
-      </c>
-      <c r="H4" s="236">
-        <f>(H3-'Metrics &amp; Drivers'!J14-'Metrics &amp; Drivers'!J20-'Metrics &amp; Drivers'!J26-'Metrics &amp; Drivers'!J32+'Metrics &amp; Drivers'!J58+8)*(1-'Metrics &amp; Drivers'!J65)</f>
-        <v>4457.8933102499996</v>
-      </c>
-      <c r="I4" s="230">
-        <f>(I3-'Metrics &amp; Drivers'!K14-'Metrics &amp; Drivers'!K20-'Metrics &amp; Drivers'!K26-'Metrics &amp; Drivers'!K32+'Metrics &amp; Drivers'!K58+8)*(1-'Metrics &amp; Drivers'!K65)</f>
-        <v>5585.7265852919991</v>
-      </c>
-      <c r="J4" s="230">
-        <f>(J3-'Metrics &amp; Drivers'!L14-'Metrics &amp; Drivers'!L20-'Metrics &amp; Drivers'!L26-'Metrics &amp; Drivers'!L32+'Metrics &amp; Drivers'!L58+8)*(1-'Metrics &amp; Drivers'!L65)</f>
-        <v>6753.2014025599992</v>
-      </c>
-      <c r="K4" s="230">
-        <f>(K3-'Metrics &amp; Drivers'!M14-'Metrics &amp; Drivers'!M20-'Metrics &amp; Drivers'!M26-'Metrics &amp; Drivers'!M32+'Metrics &amp; Drivers'!M58+8)*(1-'Metrics &amp; Drivers'!M65)</f>
-        <v>7885.9966841045753</v>
-      </c>
-      <c r="L4" s="230">
-        <f>(L3-'Metrics &amp; Drivers'!N14-'Metrics &amp; Drivers'!N20-'Metrics &amp; Drivers'!N26-'Metrics &amp; Drivers'!N32+'Metrics &amp; Drivers'!N58+8)*(1-'Metrics &amp; Drivers'!N65)</f>
-        <v>9027.0385522138695</v>
-      </c>
-      <c r="M4" s="230">
-        <f>(M3-'Metrics &amp; Drivers'!O14-'Metrics &amp; Drivers'!O20-'Metrics &amp; Drivers'!O26-'Metrics &amp; Drivers'!O32+'Metrics &amp; Drivers'!O58+8)*(1-'Metrics &amp; Drivers'!O65)</f>
-        <v>10061.968065186897</v>
-      </c>
-    </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B5" s="232" t="s">
-        <v>230</v>
-      </c>
-      <c r="C5" s="233">
-        <f>C4/C3</f>
-        <v>1.2638287207761984E-2</v>
-      </c>
-      <c r="D5" s="233">
-        <f>D4/D3</f>
-        <v>-6.8506620283270037E-2</v>
-      </c>
-      <c r="E5" s="233">
-        <f>E4/E3</f>
-        <v>0.10863817733239926</v>
-      </c>
-      <c r="F5" s="233">
-        <f>F4/F3</f>
-        <v>0.49000651344561275</v>
-      </c>
-      <c r="G5" s="233">
-        <f>G4/G3</f>
-        <v>0.6082744904847921</v>
-      </c>
-      <c r="H5" s="237">
-        <f>H4/H3</f>
-        <v>0.63794531902859131</v>
-      </c>
-      <c r="I5" s="233">
-        <f>I4/I3</f>
-        <v>0.64463187061695082</v>
-      </c>
-      <c r="J5" s="233">
-        <f>J4/J3</f>
-        <v>0.64947218389460037</v>
-      </c>
-      <c r="K5" s="233">
-        <f>K4/K3</f>
-        <v>0.65380683191916378</v>
-      </c>
-      <c r="L5" s="233">
-        <f>L4/L3</f>
-        <v>0.65649785307699227</v>
-      </c>
-      <c r="M5" s="233">
-        <f>M4/M3</f>
-        <v>0.65924670646800665</v>
-      </c>
-    </row>
-    <row r="6" spans="2:13" collapsed="1" x14ac:dyDescent="0.3"/>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4C649D4-0C72-424C-AF62-F2FC33ADC866}">
   <dimension ref="B2:I57"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -10935,15 +9400,15 @@
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B6" s="2"/>
-      <c r="C6" s="224" t="s">
+      <c r="C6" s="225" t="s">
         <v>117</v>
       </c>
-      <c r="D6" s="224"/>
-      <c r="E6" s="224"/>
-      <c r="F6" s="224"/>
-      <c r="G6" s="224"/>
-      <c r="H6" s="224"/>
-      <c r="I6" s="224"/>
+      <c r="D6" s="225"/>
+      <c r="E6" s="225"/>
+      <c r="F6" s="225"/>
+      <c r="G6" s="225"/>
+      <c r="H6" s="225"/>
+      <c r="I6" s="225"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B7" s="216"/>
@@ -12135,4 +10600,1208 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1B8D43B-0AE5-451E-8577-8383133CC245}">
+  <dimension ref="B2:I53"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="1.88671875" customWidth="1"/>
+    <col min="2" max="2" width="46.33203125" customWidth="1"/>
+    <col min="3" max="9" width="15.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:9" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="B2" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B3" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B6" s="2"/>
+      <c r="C6" s="225" t="s">
+        <v>117</v>
+      </c>
+      <c r="D6" s="225"/>
+      <c r="E6" s="225"/>
+      <c r="F6" s="225"/>
+      <c r="G6" s="225"/>
+      <c r="H6" s="225"/>
+      <c r="I6" s="225"/>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B7" s="216"/>
+      <c r="C7" s="216">
+        <v>2019</v>
+      </c>
+      <c r="D7" s="216">
+        <v>2020</v>
+      </c>
+      <c r="E7" s="216">
+        <v>2021</v>
+      </c>
+      <c r="F7" s="216">
+        <v>2022</v>
+      </c>
+      <c r="G7" s="216">
+        <v>2023</v>
+      </c>
+      <c r="H7" s="216">
+        <v>2024</v>
+      </c>
+      <c r="I7" s="216">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B8" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B9" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C9" s="16">
+        <f>'Income Statement'!C29</f>
+        <v>118.99999999999994</v>
+      </c>
+      <c r="D9" s="16">
+        <f>'Income Statement'!D29</f>
+        <v>-43.320000000000192</v>
+      </c>
+      <c r="E9" s="16">
+        <f>'Income Statement'!E29</f>
+        <v>35.29999999999977</v>
+      </c>
+      <c r="F9" s="16">
+        <f>'Income Statement'!F29</f>
+        <v>-192.98999999999998</v>
+      </c>
+      <c r="G9" s="16">
+        <f>'Income Statement'!G29</f>
+        <v>356.66999999999979</v>
+      </c>
+      <c r="H9" s="16">
+        <f>'Income Statement'!H29</f>
+        <v>1579.83</v>
+      </c>
+      <c r="I9" s="16">
+        <f>'Income Statement'!I29</f>
+        <v>3333.77</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B10" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B11" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C11" s="6">
+        <v>92.81</v>
+      </c>
+      <c r="D11" s="6">
+        <v>255</v>
+      </c>
+      <c r="E11" s="6">
+        <v>431.1</v>
+      </c>
+      <c r="F11" s="6">
+        <v>547.1</v>
+      </c>
+      <c r="G11" s="6">
+        <v>489</v>
+      </c>
+      <c r="H11" s="6">
+        <v>448.7</v>
+      </c>
+      <c r="I11" s="6">
+        <v>194.8</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B12" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C12" s="6">
+        <v>10.220000000000001</v>
+      </c>
+      <c r="D12" s="6">
+        <v>62.39</v>
+      </c>
+      <c r="E12" s="6">
+        <v>133.19999999999999</v>
+      </c>
+      <c r="F12" s="6">
+        <v>191.6</v>
+      </c>
+      <c r="G12" s="6">
+        <v>363.1</v>
+      </c>
+      <c r="H12" s="6">
+        <v>369.4</v>
+      </c>
+      <c r="I12" s="6">
+        <v>210.4</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B13" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C13" s="6">
+        <v>4.9800000000000004</v>
+      </c>
+      <c r="D13" s="6">
+        <v>8.15</v>
+      </c>
+      <c r="E13" s="6">
+        <v>12.83</v>
+      </c>
+      <c r="F13" s="6">
+        <v>12.68</v>
+      </c>
+      <c r="G13" s="6">
+        <v>9.36</v>
+      </c>
+      <c r="H13" s="6">
+        <v>5.46</v>
+      </c>
+      <c r="I13" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B14" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C14" s="6">
+        <v>0</v>
+      </c>
+      <c r="D14" s="6">
+        <v>0</v>
+      </c>
+      <c r="E14" s="6">
+        <v>0</v>
+      </c>
+      <c r="F14" s="6">
+        <v>0</v>
+      </c>
+      <c r="G14" s="6">
+        <v>0</v>
+      </c>
+      <c r="H14" s="6">
+        <v>0</v>
+      </c>
+      <c r="I14" s="6">
+        <v>188.9</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B15" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C15" s="6">
+        <v>0</v>
+      </c>
+      <c r="D15" s="6">
+        <v>0</v>
+      </c>
+      <c r="E15" s="6">
+        <v>0</v>
+      </c>
+      <c r="F15" s="6">
+        <v>0</v>
+      </c>
+      <c r="G15" s="6">
+        <v>0</v>
+      </c>
+      <c r="H15" s="6">
+        <v>0</v>
+      </c>
+      <c r="I15" s="6">
+        <v>-106.2</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B16" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C16" s="6">
+        <v>0</v>
+      </c>
+      <c r="D16" s="6">
+        <v>0</v>
+      </c>
+      <c r="E16" s="6">
+        <v>0</v>
+      </c>
+      <c r="F16" s="6">
+        <v>0</v>
+      </c>
+      <c r="G16" s="6">
+        <v>27.95</v>
+      </c>
+      <c r="H16" s="6">
+        <v>0</v>
+      </c>
+      <c r="I16" s="6">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B17" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C17" s="6">
+        <v>0</v>
+      </c>
+      <c r="D17" s="6">
+        <v>0</v>
+      </c>
+      <c r="E17" s="6">
+        <v>0</v>
+      </c>
+      <c r="F17" s="6">
+        <v>127.9</v>
+      </c>
+      <c r="G17" s="6">
+        <v>0</v>
+      </c>
+      <c r="H17" s="6">
+        <v>1.65</v>
+      </c>
+      <c r="I17" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B18" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0</v>
+      </c>
+      <c r="D18" s="6">
+        <v>0</v>
+      </c>
+      <c r="E18" s="6">
+        <v>18.239999999999998</v>
+      </c>
+      <c r="F18" s="6">
+        <v>0</v>
+      </c>
+      <c r="G18" s="6">
+        <v>0</v>
+      </c>
+      <c r="H18" s="6">
+        <v>28.38</v>
+      </c>
+      <c r="I18" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B19" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C19" s="6">
+        <v>2.69</v>
+      </c>
+      <c r="D19" s="6">
+        <v>7.68</v>
+      </c>
+      <c r="E19" s="6">
+        <v>15.58</v>
+      </c>
+      <c r="F19" s="6">
+        <v>18.91</v>
+      </c>
+      <c r="G19" s="6">
+        <v>24.13</v>
+      </c>
+      <c r="H19" s="6">
+        <v>15.06</v>
+      </c>
+      <c r="I19" s="6">
+        <v>21.46</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B20" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B21" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C21" s="6">
+        <v>-33.520000000000003</v>
+      </c>
+      <c r="D21" s="6">
+        <v>-113.2</v>
+      </c>
+      <c r="E21" s="6">
+        <v>-202</v>
+      </c>
+      <c r="F21" s="6">
+        <v>-174.8</v>
+      </c>
+      <c r="G21" s="6">
+        <v>-261.3</v>
+      </c>
+      <c r="H21" s="6">
+        <v>-467</v>
+      </c>
+      <c r="I21" s="6">
+        <v>-542.20000000000005</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B22" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C22" s="6">
+        <v>-21.35</v>
+      </c>
+      <c r="D22" s="6">
+        <v>-32.380000000000003</v>
+      </c>
+      <c r="E22" s="6">
+        <v>-143.26</v>
+      </c>
+      <c r="F22" s="6">
+        <v>-81.06</v>
+      </c>
+      <c r="G22" s="6">
+        <v>-133.97999999999999</v>
+      </c>
+      <c r="H22" s="6">
+        <v>-185.34</v>
+      </c>
+      <c r="I22" s="6">
+        <v>134.69999999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B23" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C23" s="6">
+        <v>13.53</v>
+      </c>
+      <c r="D23" s="6">
+        <v>49.12</v>
+      </c>
+      <c r="E23" s="6">
+        <v>98.61</v>
+      </c>
+      <c r="F23" s="6">
+        <v>3.48</v>
+      </c>
+      <c r="G23" s="6">
+        <v>98.57</v>
+      </c>
+      <c r="H23" s="6">
+        <v>189.6</v>
+      </c>
+      <c r="I23" s="6">
+        <v>232.5</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B24" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C24" s="6">
+        <v>5.66</v>
+      </c>
+      <c r="D24" s="6">
+        <v>2.78</v>
+      </c>
+      <c r="E24" s="6">
+        <v>3.06</v>
+      </c>
+      <c r="F24" s="6">
+        <v>-6.41</v>
+      </c>
+      <c r="G24" s="6">
+        <v>92.75</v>
+      </c>
+      <c r="H24" s="6">
+        <v>134</v>
+      </c>
+      <c r="I24" s="6">
+        <v>268.2</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B25" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C25" s="6">
+        <v>6.72</v>
+      </c>
+      <c r="D25" s="6">
+        <v>35.49</v>
+      </c>
+      <c r="E25" s="6">
+        <v>-13.91</v>
+      </c>
+      <c r="F25" s="6">
+        <v>-14.71</v>
+      </c>
+      <c r="G25" s="6">
+        <v>13.86</v>
+      </c>
+      <c r="H25" s="6">
+        <v>-6.63</v>
+      </c>
+      <c r="I25" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B26" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C26" s="6">
+        <v>-2.2400000000000002</v>
+      </c>
+      <c r="D26" s="6">
+        <v>-8.81</v>
+      </c>
+      <c r="E26" s="6">
+        <v>-26.85</v>
+      </c>
+      <c r="F26" s="6">
+        <v>-18.899999999999999</v>
+      </c>
+      <c r="G26" s="6">
+        <v>-18.61</v>
+      </c>
+      <c r="H26" s="6">
+        <v>-14.11</v>
+      </c>
+      <c r="I26" s="6">
+        <v>-15.23</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B27" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C27" s="7">
+        <f>C9+SUM(C11:C19)+SUM(C21:C26)</f>
+        <v>198.49999999999991</v>
+      </c>
+      <c r="D27" s="7">
+        <f t="shared" ref="D27:I27" si="0">D9+SUM(D11:D19)+SUM(D21:D26)</f>
+        <v>222.89999999999975</v>
+      </c>
+      <c r="E27" s="7">
+        <f t="shared" si="0"/>
+        <v>361.89999999999975</v>
+      </c>
+      <c r="F27" s="7">
+        <f t="shared" si="0"/>
+        <v>412.79999999999995</v>
+      </c>
+      <c r="G27" s="7">
+        <f t="shared" si="0"/>
+        <v>1061.4999999999998</v>
+      </c>
+      <c r="H27" s="7">
+        <f t="shared" si="0"/>
+        <v>2098.9999999999995</v>
+      </c>
+      <c r="I27" s="7">
+        <f t="shared" si="0"/>
+        <v>3971.1</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B28" s="2"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
+      <c r="H28" s="8"/>
+      <c r="I28" s="8"/>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B29" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="8"/>
+      <c r="I29" s="8"/>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B30" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C30" s="6">
+        <v>-404.2</v>
+      </c>
+      <c r="D30" s="6">
+        <v>-674.7</v>
+      </c>
+      <c r="E30" s="6">
+        <v>-1206.5</v>
+      </c>
+      <c r="F30" s="6">
+        <v>-1339.8</v>
+      </c>
+      <c r="G30" s="6">
+        <v>0</v>
+      </c>
+      <c r="H30" s="6">
+        <v>0</v>
+      </c>
+      <c r="I30" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B31" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C31" s="6">
+        <v>-3.36</v>
+      </c>
+      <c r="D31" s="6">
+        <v>-3.24</v>
+      </c>
+      <c r="E31" s="6">
+        <v>-1.39</v>
+      </c>
+      <c r="F31" s="6">
+        <v>-0.66</v>
+      </c>
+      <c r="G31" s="6">
+        <v>-4.25</v>
+      </c>
+      <c r="H31" s="6">
+        <v>-4.78</v>
+      </c>
+      <c r="I31" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B32" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C32" s="6">
+        <v>0</v>
+      </c>
+      <c r="D32" s="6">
+        <v>0</v>
+      </c>
+      <c r="E32" s="6">
+        <v>-4.07</v>
+      </c>
+      <c r="F32" s="6">
+        <v>-5.95</v>
+      </c>
+      <c r="G32" s="6">
+        <v>-63.9</v>
+      </c>
+      <c r="H32" s="6">
+        <v>-25.55</v>
+      </c>
+      <c r="I32" s="6">
+        <v>-28.32</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B33" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C33" s="6">
+        <v>-4</v>
+      </c>
+      <c r="D33" s="6">
+        <v>-2</v>
+      </c>
+      <c r="E33" s="6">
+        <v>-15</v>
+      </c>
+      <c r="F33" s="6">
+        <v>-66.34</v>
+      </c>
+      <c r="G33" s="6">
+        <v>-17.93</v>
+      </c>
+      <c r="H33" s="6">
+        <v>-76.98</v>
+      </c>
+      <c r="I33" s="6">
+        <v>-20.18</v>
+      </c>
+    </row>
+    <row r="34" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B34" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C34" s="6">
+        <v>0</v>
+      </c>
+      <c r="D34" s="6">
+        <v>0</v>
+      </c>
+      <c r="E34" s="6">
+        <v>12.01</v>
+      </c>
+      <c r="F34" s="6">
+        <v>41.31</v>
+      </c>
+      <c r="G34" s="6">
+        <v>8.25</v>
+      </c>
+      <c r="H34" s="6">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="I34" s="6">
+        <v>407.3</v>
+      </c>
+    </row>
+    <row r="35" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B35" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C35" s="6">
+        <v>-0.04</v>
+      </c>
+      <c r="D35" s="6">
+        <v>0.04</v>
+      </c>
+      <c r="E35" s="6">
+        <v>0.05</v>
+      </c>
+      <c r="F35" s="6">
+        <v>-0.06</v>
+      </c>
+      <c r="G35" s="6">
+        <v>0</v>
+      </c>
+      <c r="H35" s="6">
+        <v>-0.05</v>
+      </c>
+      <c r="I35" s="6">
+        <v>-0.4</v>
+      </c>
+    </row>
+    <row r="36" spans="2:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B36" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C36" s="7">
+        <f>SUM(C30:C35)</f>
+        <v>-411.6</v>
+      </c>
+      <c r="D36" s="7">
+        <f t="shared" ref="D36:I36" si="1">SUM(D30:D35)</f>
+        <v>-679.90000000000009</v>
+      </c>
+      <c r="E36" s="7">
+        <f t="shared" si="1"/>
+        <v>-1214.9000000000001</v>
+      </c>
+      <c r="F36" s="7">
+        <f t="shared" si="1"/>
+        <v>-1371.5</v>
+      </c>
+      <c r="G36" s="7">
+        <f t="shared" si="1"/>
+        <v>-77.830000000000013</v>
+      </c>
+      <c r="H36" s="7">
+        <f t="shared" si="1"/>
+        <v>-106.8</v>
+      </c>
+      <c r="I36" s="7">
+        <f t="shared" si="1"/>
+        <v>358.40000000000003</v>
+      </c>
+    </row>
+    <row r="37" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B37" s="2"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+      <c r="G37" s="8"/>
+      <c r="H37" s="8"/>
+      <c r="I37" s="8"/>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B38" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="8"/>
+      <c r="H38" s="8"/>
+      <c r="I38" s="8"/>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B39" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C39" s="6">
+        <v>388.9</v>
+      </c>
+      <c r="D39" s="6">
+        <v>481.3</v>
+      </c>
+      <c r="E39" s="6">
+        <v>2329.1</v>
+      </c>
+      <c r="F39" s="6">
+        <v>0</v>
+      </c>
+      <c r="G39" s="6">
+        <v>395.3</v>
+      </c>
+      <c r="H39" s="6">
+        <v>4614.8</v>
+      </c>
+      <c r="I39" s="6">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B40" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C40" s="6">
+        <v>-11.21</v>
+      </c>
+      <c r="D40" s="6">
+        <v>-64.290000000000006</v>
+      </c>
+      <c r="E40" s="6">
+        <v>-719.8</v>
+      </c>
+      <c r="F40" s="6">
+        <v>-25.81</v>
+      </c>
+      <c r="G40" s="6">
+        <v>-498</v>
+      </c>
+      <c r="H40" s="6">
+        <v>-4225.2</v>
+      </c>
+      <c r="I40" s="6">
+        <v>-200</v>
+      </c>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B41" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C41" s="6">
+        <v>-0.01</v>
+      </c>
+      <c r="D41" s="6">
+        <v>-1.77</v>
+      </c>
+      <c r="E41" s="6">
+        <v>0</v>
+      </c>
+      <c r="F41" s="6">
+        <v>-338.9</v>
+      </c>
+      <c r="G41" s="6">
+        <v>-1153.5999999999999</v>
+      </c>
+      <c r="H41" s="6">
+        <v>-981.3</v>
+      </c>
+      <c r="I41" s="6">
+        <v>-2191.9</v>
+      </c>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B42" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C42" s="6">
+        <v>0</v>
+      </c>
+      <c r="D42" s="6">
+        <v>0</v>
+      </c>
+      <c r="E42" s="6">
+        <v>0</v>
+      </c>
+      <c r="F42" s="6">
+        <v>-27.53</v>
+      </c>
+      <c r="G42" s="6">
+        <v>-246.4</v>
+      </c>
+      <c r="H42" s="6">
+        <v>-1143.5</v>
+      </c>
+      <c r="I42" s="6">
+        <v>-392.4</v>
+      </c>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B43" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C43" s="6">
+        <v>2.64</v>
+      </c>
+      <c r="D43" s="6">
+        <v>11.62</v>
+      </c>
+      <c r="E43" s="6">
+        <v>1779.24</v>
+      </c>
+      <c r="F43" s="6">
+        <v>31.02</v>
+      </c>
+      <c r="G43" s="6">
+        <v>25.79</v>
+      </c>
+      <c r="H43" s="6">
+        <v>41.8</v>
+      </c>
+      <c r="I43" s="6">
+        <v>25.33</v>
+      </c>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B44" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C44" s="6">
+        <v>-5.66</v>
+      </c>
+      <c r="D44" s="6">
+        <v>-9.7100000000000009</v>
+      </c>
+      <c r="E44" s="6">
+        <v>-15.27</v>
+      </c>
+      <c r="F44" s="6">
+        <v>-24.08</v>
+      </c>
+      <c r="G44" s="6">
+        <v>-20.170000000000002</v>
+      </c>
+      <c r="H44" s="6">
+        <v>-20.87</v>
+      </c>
+      <c r="I44" s="6">
+        <v>-18.670000000000002</v>
+      </c>
+    </row>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B45" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C45" s="6">
+        <v>-41.46</v>
+      </c>
+      <c r="D45" s="6">
+        <v>-39.25</v>
+      </c>
+      <c r="E45" s="6">
+        <v>-263.67</v>
+      </c>
+      <c r="F45" s="6">
+        <v>-141.6</v>
+      </c>
+      <c r="G45" s="6">
+        <v>-65.72</v>
+      </c>
+      <c r="H45" s="6">
+        <v>-35.53</v>
+      </c>
+      <c r="I45" s="6">
+        <v>-15.46</v>
+      </c>
+    </row>
+    <row r="46" spans="2:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B46" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C46" s="7">
+        <f>SUM(C39:C45)</f>
+        <v>333.2</v>
+      </c>
+      <c r="D46" s="7">
+        <f t="shared" ref="D46:I46" si="2">SUM(D39:D45)</f>
+        <v>377.90000000000003</v>
+      </c>
+      <c r="E46" s="7">
+        <f t="shared" si="2"/>
+        <v>3109.6</v>
+      </c>
+      <c r="F46" s="7">
+        <f t="shared" si="2"/>
+        <v>-526.9</v>
+      </c>
+      <c r="G46" s="7">
+        <f t="shared" si="2"/>
+        <v>-1562.8000000000002</v>
+      </c>
+      <c r="H46" s="7">
+        <f t="shared" si="2"/>
+        <v>-1749.7999999999995</v>
+      </c>
+      <c r="I46" s="7">
+        <f t="shared" si="2"/>
+        <v>-2593.1000000000004</v>
+      </c>
+    </row>
+    <row r="47" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B47" s="2"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="8"/>
+      <c r="E47" s="8"/>
+      <c r="F47" s="8"/>
+      <c r="G47" s="8"/>
+      <c r="H47" s="8"/>
+      <c r="I47" s="8"/>
+    </row>
+    <row r="48" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B48" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C48" s="6">
+        <v>0.06</v>
+      </c>
+      <c r="D48" s="6">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="E48" s="6">
+        <v>-3.2</v>
+      </c>
+      <c r="F48" s="6">
+        <v>-4.4800000000000004</v>
+      </c>
+      <c r="G48" s="6">
+        <v>0.78</v>
+      </c>
+      <c r="H48" s="6">
+        <v>-3.15</v>
+      </c>
+      <c r="I48" s="6">
+        <v>9.23</v>
+      </c>
+    </row>
+    <row r="49" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B49" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C49" s="6">
+        <v>0</v>
+      </c>
+      <c r="D49" s="6">
+        <v>0</v>
+      </c>
+      <c r="E49" s="6">
+        <v>0</v>
+      </c>
+      <c r="F49" s="6">
+        <v>0</v>
+      </c>
+      <c r="G49" s="6">
+        <v>0</v>
+      </c>
+      <c r="H49" s="6">
+        <v>0</v>
+      </c>
+      <c r="I49" s="6">
+        <v>44.38</v>
+      </c>
+    </row>
+    <row r="50" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B50" s="2"/>
+      <c r="C50" s="8"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8"/>
+      <c r="F50" s="8"/>
+      <c r="G50" s="8"/>
+      <c r="H50" s="8"/>
+      <c r="I50" s="8"/>
+    </row>
+    <row r="51" spans="2:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B51" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C51" s="7">
+        <f>C27+C36+C46+C48+C49</f>
+        <v>120.15999999999988</v>
+      </c>
+      <c r="D51" s="7">
+        <f t="shared" ref="D51:I51" si="3">D27+D36+D46+D48+D49</f>
+        <v>-78.960000000000306</v>
+      </c>
+      <c r="E51" s="7">
+        <f t="shared" si="3"/>
+        <v>2253.3999999999996</v>
+      </c>
+      <c r="F51" s="7">
+        <f t="shared" si="3"/>
+        <v>-1490.08</v>
+      </c>
+      <c r="G51" s="7">
+        <f t="shared" si="3"/>
+        <v>-578.35000000000048</v>
+      </c>
+      <c r="H51" s="7">
+        <f t="shared" si="3"/>
+        <v>239.25000000000009</v>
+      </c>
+      <c r="I51" s="7">
+        <f t="shared" si="3"/>
+        <v>1790.0099999999998</v>
+      </c>
+    </row>
+    <row r="52" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B52" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C52" s="6">
+        <v>276.10000000000002</v>
+      </c>
+      <c r="D52" s="6">
+        <v>396.3</v>
+      </c>
+      <c r="E52" s="6">
+        <v>317.2</v>
+      </c>
+      <c r="F52" s="6">
+        <v>2570.5</v>
+      </c>
+      <c r="G52" s="6">
+        <v>1080.5</v>
+      </c>
+      <c r="H52" s="6">
+        <v>502.2</v>
+      </c>
+      <c r="I52" s="6">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="53" spans="2:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B53" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C53" s="7">
+        <f>C52+C51</f>
+        <v>396.25999999999988</v>
+      </c>
+      <c r="D53" s="7">
+        <f t="shared" ref="D53:I53" si="4">D52+D51</f>
+        <v>317.33999999999969</v>
+      </c>
+      <c r="E53" s="7">
+        <f t="shared" si="4"/>
+        <v>2570.5999999999995</v>
+      </c>
+      <c r="F53" s="7">
+        <f t="shared" si="4"/>
+        <v>1080.42</v>
+      </c>
+      <c r="G53" s="7">
+        <f t="shared" si="4"/>
+        <v>502.14999999999952</v>
+      </c>
+      <c r="H53" s="7">
+        <f t="shared" si="4"/>
+        <v>741.45</v>
+      </c>
+      <c r="I53" s="7">
+        <f t="shared" si="4"/>
+        <v>2487.0099999999998</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C6:I6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>